<commit_message>
Roster cleanup: enroll/remove/track-fix scripts, HRA templates, suppress future-year at-risk
</commit_message>
<xml_diff>
--- a/task_templates_starter.xlsx
+++ b/task_templates_starter.xlsx
@@ -482,9 +482,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -499,9 +497,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -544,9 +540,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
@@ -638,9 +632,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
@@ -690,9 +682,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-    </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
@@ -739,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M87"/>
+  <dimension ref="A1:M96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6067,6 +6057,546 @@
       <c r="M87" s="5" t="inlineStr">
         <is>
           <t>Sustainability hospitals submit one quarter's worth of data per year. Quarter is configurable per hospital; default Q1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>SOAR</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>sustainability</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Sustainability Q1</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Complete bi-annual 1:1 QI advising (first half) — early</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>qi_advising</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>quarterly</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>End of March</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>Either this Q1 task OR the Q2 task fulfills the first-half advising requirement. SOAR sustainability requires one advising session in Jan–June and one in Jul–Dec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>TTT</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Implementation Q1</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Complete Q1 Hospital Readiness Assessment</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>readiness_assessment</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>quarterly</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>End of March</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>HRA submitted via REDCap; we only track that it was completed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>TTT</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Implementation Q4</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Complete Q4 Hospital Readiness Assessment</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>readiness_assessment</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>quarterly</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>End of December</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>HRA submitted via REDCap; we only track that it was completed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>NEST</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Implementation Q1</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Complete Q1 Hospital Readiness Assessment</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>readiness_assessment</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>quarterly</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>End of March</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>HRA submitted via REDCap; we only track that it was completed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>NEST</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Implementation Q4</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Complete Q4 Hospital Readiness Assessment</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>readiness_assessment</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>quarterly</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>End of December</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>HRA submitted via REDCap; we only track that it was completed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>SOAR</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Implementation Q1</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Complete Q1 Hospital Readiness Assessment</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>readiness_assessment</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>quarterly</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>End of March</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>HRA submitted via REDCap; we only track that it was completed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>SOAR</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Implementation Q4</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Complete Q4 Hospital Readiness Assessment</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>readiness_assessment</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>quarterly</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>End of December</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>HRA submitted via REDCap; we only track that it was completed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>SPARK</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Implementation Q2</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Complete Q2 Hospital Readiness Assessment</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>readiness_assessment</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>quarterly</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>End of June</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>HRA submitted via REDCap. 2026 SPARK schedule is Q2 + Q4 (not the standard Q1 + Q4) — update templates before 2027 cohort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>SPARK</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Implementation Q4</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Complete Q4 Hospital Readiness Assessment</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>readiness_assessment</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>quarterly</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>End of December</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>HRA submitted via REDCap. 2026 SPARK schedule is Q2 + Q4 — see Notes on Q2 row.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: SOAR sustainability QI advising is bi-annual (2 tasks, not 3)
CPCQC's sustainability requirement is one 1:1 QI advising session in the
first half of the year (deadline Jun 30) and one in the second half
(deadline Dec 31) — TWO tasks per year. The templates spreadsheet had a
stray "Complete bi-annual 1:1 QI advising (first half) — early" row
labeled Q1, which spawned an extra task instance per SOAR sustainability
hospital. It never counted toward the required 2 of 2 (the compliance
engine has always used Q2+Q4 via defaultAdvisingQuarters(2)), but it
cluttered the task overview with a Q1 row showing "Not started" all year.

- Remove the early row from task_templates_starter.xlsx.
- Migration 0014 deletes the template and every TaskInstance it spawned.
- Drop the stale "new Q1 advising for SOAR sustainability" mention in
  the backfill script's docstring.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/task_templates_starter.xlsx
+++ b/task_templates_starter.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TaskTemplates" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StageDefinitions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meetings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TaskTemplates" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="StageDefinitions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Requirements" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Meetings" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -724,7 +724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M128"/>
+  <dimension ref="A1:M127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5081,36 +5081,36 @@
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SOAR</t>
+          <t>TTT</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>sustainability</t>
+          <t>active</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Sustainability Q1</t>
+          <t>Implementation Q1</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Complete bi-annual 1:1 QI advising (first half) — early</t>
+          <t>Complete Q1 Hospital Readiness Assessment</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>qi_advising</t>
+          <t>readiness_assessment</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -5135,13 +5135,13 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>Either this Q1 task OR the Q2 task fulfills the first-half advising requirement. SOAR sustainability requires one advising session in Jan–June and one in Jul–Dec.</t>
+          <t>HRA submitted via REDCap; we only track that it was completed.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -5155,17 +5155,17 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Implementation Q1</t>
+          <t>Implementation Q4</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Complete Q1 Hospital Readiness Assessment</t>
+          <t>Complete Q4 Hospital Readiness Assessment</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -5180,12 +5180,12 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>End of March</t>
+          <t>End of December</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5201,11 +5201,11 @@
     </row>
     <row r="74" ht="30" customHeight="1">
       <c r="A74" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>TTT</t>
+          <t>NEST</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -5215,17 +5215,17 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Implementation Q4</t>
+          <t>Implementation Q1</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Complete Q4 Hospital Readiness Assessment</t>
+          <t>Complete Q1 Hospital Readiness Assessment</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -5240,12 +5240,12 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>End of December</t>
+          <t>End of March</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5261,7 +5261,7 @@
     </row>
     <row r="75" ht="30" customHeight="1">
       <c r="A75" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -5275,17 +5275,17 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Implementation Q1</t>
+          <t>Implementation Q4</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Complete Q1 Hospital Readiness Assessment</t>
+          <t>Complete Q4 Hospital Readiness Assessment</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -5300,12 +5300,12 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>End of March</t>
+          <t>End of December</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5321,11 +5321,11 @@
     </row>
     <row r="76" ht="30" customHeight="1">
       <c r="A76" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>NEST</t>
+          <t>SOAR</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -5335,17 +5335,17 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Implementation Q4</t>
+          <t>Implementation Q1</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Complete Q4 Hospital Readiness Assessment</t>
+          <t>Complete Q1 Hospital Readiness Assessment</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -5360,12 +5360,12 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>End of December</t>
+          <t>End of March</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5381,7 +5381,7 @@
     </row>
     <row r="77" ht="30" customHeight="1">
       <c r="A77" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -5395,17 +5395,17 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Implementation Q1</t>
+          <t>Implementation Q4</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Complete Q1 Hospital Readiness Assessment</t>
+          <t>Complete Q4 Hospital Readiness Assessment</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -5420,12 +5420,12 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>End of March</t>
+          <t>End of December</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5441,11 +5441,11 @@
     </row>
     <row r="78" ht="30" customHeight="1">
       <c r="A78" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SOAR</t>
+          <t>SPARK</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -5455,17 +5455,17 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Implementation Q4</t>
+          <t>Implementation Q2</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Complete Q4 Hospital Readiness Assessment</t>
+          <t>Complete Q2 Hospital Readiness Assessment</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -5480,12 +5480,12 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>End of December</t>
+          <t>End of June</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5495,13 +5495,13 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>HRA submitted via REDCap; we only track that it was completed.</t>
+          <t>HRA submitted via REDCap. 2026 SPARK schedule is Q2 + Q4 (not the standard Q1 + Q4) — update templates before 2027 cohort.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="30" customHeight="1">
       <c r="A79" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -5515,17 +5515,17 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Implementation Q2</t>
+          <t>Implementation Q4</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Complete Q2 Hospital Readiness Assessment</t>
+          <t>Complete Q4 Hospital Readiness Assessment</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -5540,12 +5540,12 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>End of June</t>
+          <t>End of December</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5555,17 +5555,17 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>HRA submitted via REDCap. 2026 SPARK schedule is Q2 + Q4 (not the standard Q1 + Q4) — update templates before 2027 cohort.</t>
+          <t>HRA submitted via REDCap. 2026 SPARK schedule is Q2 + Q4 — see Notes on Q2 row.</t>
         </is>
       </c>
     </row>
     <row r="80" ht="30" customHeight="1">
       <c r="A80" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SPARK</t>
+          <t>TTT</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -5575,37 +5575,37 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Implementation Q4</t>
+          <t>Implementation Q1</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Complete Q4 Hospital Readiness Assessment</t>
+          <t>Attend the January TTT initiative meeting</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>readiness_assessment</t>
+          <t>meeting_attendance</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>quarterly</t>
+          <t>monthly</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>January</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>End of December</t>
+          <t>End of January</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5615,13 +5615,13 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>HRA submitted via REDCap. 2026 SPARK schedule is Q2 + Q4 — see Notes on Q2 row.</t>
+          <t>Annual requirement: at least 9 of 12 monthly meetings. Annual Forum attendance counts toward the month it falls in (September in 2026).</t>
         </is>
       </c>
     </row>
     <row r="81" ht="30" customHeight="1">
       <c r="A81" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -5645,7 +5645,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Attend the January TTT initiative meeting</t>
+          <t>Attend the February TTT initiative meeting</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -5660,12 +5660,12 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>January</t>
+          <t>February</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>End of January</t>
+          <t>End of February</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5681,7 +5681,7 @@
     </row>
     <row r="82" ht="30" customHeight="1">
       <c r="A82" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -5705,7 +5705,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Attend the February TTT initiative meeting</t>
+          <t>Attend the March TTT initiative meeting</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -5720,12 +5720,12 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>February</t>
+          <t>March</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>End of February</t>
+          <t>End of March</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5741,7 +5741,7 @@
     </row>
     <row r="83" ht="30" customHeight="1">
       <c r="A83" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -5755,17 +5755,17 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Implementation Q1</t>
+          <t>Implementation Q2</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Attend the March TTT initiative meeting</t>
+          <t>Attend the April TTT initiative meeting</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -5780,12 +5780,12 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>March</t>
+          <t>April</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>End of March</t>
+          <t>End of April</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5801,7 +5801,7 @@
     </row>
     <row r="84" ht="30" customHeight="1">
       <c r="A84" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -5825,7 +5825,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Attend the April TTT initiative meeting</t>
+          <t>Attend the May TTT initiative meeting</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -5840,12 +5840,12 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>April</t>
+          <t>May</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>End of April</t>
+          <t>End of May</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5861,7 +5861,7 @@
     </row>
     <row r="85" ht="30" customHeight="1">
       <c r="A85" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -5885,7 +5885,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Attend the May TTT initiative meeting</t>
+          <t>Attend the June TTT initiative meeting</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -5900,12 +5900,12 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>June</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>End of May</t>
+          <t>End of June</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5921,7 +5921,7 @@
     </row>
     <row r="86" ht="30" customHeight="1">
       <c r="A86" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -5935,17 +5935,17 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Implementation Q2</t>
+          <t>Implementation Q3</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Attend the June TTT initiative meeting</t>
+          <t>Attend the July TTT initiative meeting</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -5960,12 +5960,12 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>June</t>
+          <t>July</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>End of June</t>
+          <t>End of July</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5981,7 +5981,7 @@
     </row>
     <row r="87" ht="30" customHeight="1">
       <c r="A87" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -6005,7 +6005,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Attend the July TTT initiative meeting</t>
+          <t>Attend the August TTT initiative meeting</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -6020,12 +6020,12 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>July</t>
+          <t>August</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>End of July</t>
+          <t>End of August</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6041,7 +6041,7 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -6065,7 +6065,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Attend the August TTT initiative meeting</t>
+          <t>Attend the September TTT initiative meeting</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -6080,12 +6080,12 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>September</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>End of August</t>
+          <t>End of September</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6101,7 +6101,7 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -6115,17 +6115,17 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Implementation Q3</t>
+          <t>Implementation Q4</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Attend the September TTT initiative meeting</t>
+          <t>Attend the October TTT initiative meeting</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -6140,12 +6140,12 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>October</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>End of September</t>
+          <t>End of October</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6161,7 +6161,7 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -6185,7 +6185,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Attend the October TTT initiative meeting</t>
+          <t>Attend the November TTT initiative meeting</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -6200,12 +6200,12 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>November</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>End of October</t>
+          <t>End of November</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6221,7 +6221,7 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -6245,7 +6245,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Attend the November TTT initiative meeting</t>
+          <t>Attend the December TTT initiative meeting</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -6260,12 +6260,12 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>November</t>
+          <t>December</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>End of November</t>
+          <t>End of December</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6281,11 +6281,11 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TTT</t>
+          <t>SPARK</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -6295,17 +6295,17 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Implementation Q4</t>
+          <t>Implementation Q1</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Attend the December TTT initiative meeting</t>
+          <t>Attend the January SPARK initiative meeting</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -6320,12 +6320,12 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>December</t>
+          <t>January</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>End of December</t>
+          <t>End of January</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6341,7 +6341,7 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -6365,7 +6365,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Attend the January SPARK initiative meeting</t>
+          <t>Attend the February SPARK initiative meeting</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -6380,12 +6380,12 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>January</t>
+          <t>February</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>End of January</t>
+          <t>End of February</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6401,7 +6401,7 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -6425,7 +6425,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Attend the February SPARK initiative meeting</t>
+          <t>Attend the March SPARK initiative meeting</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -6440,12 +6440,12 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>February</t>
+          <t>March</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>End of February</t>
+          <t>End of March</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6461,7 +6461,7 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -6475,17 +6475,17 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Implementation Q1</t>
+          <t>Implementation Q2</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Attend the March SPARK initiative meeting</t>
+          <t>Attend the April SPARK initiative meeting</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -6500,12 +6500,12 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>March</t>
+          <t>April</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>End of March</t>
+          <t>End of April</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6521,7 +6521,7 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -6545,7 +6545,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Attend the April SPARK initiative meeting</t>
+          <t>Attend the May SPARK initiative meeting</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -6560,12 +6560,12 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>April</t>
+          <t>May</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>End of April</t>
+          <t>End of May</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6581,7 +6581,7 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -6605,7 +6605,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Attend the May SPARK initiative meeting</t>
+          <t>Attend the June SPARK initiative meeting</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -6620,12 +6620,12 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>June</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>End of May</t>
+          <t>End of June</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6641,7 +6641,7 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -6655,17 +6655,17 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Implementation Q2</t>
+          <t>Implementation Q3</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Attend the June SPARK initiative meeting</t>
+          <t>Attend the July SPARK initiative meeting</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -6680,12 +6680,12 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>June</t>
+          <t>July</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>End of June</t>
+          <t>End of July</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6701,7 +6701,7 @@
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -6725,7 +6725,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Attend the July SPARK initiative meeting</t>
+          <t>Attend the August SPARK initiative meeting</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -6740,12 +6740,12 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>July</t>
+          <t>August</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>End of July</t>
+          <t>End of August</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6761,7 +6761,7 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -6785,7 +6785,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Attend the August SPARK initiative meeting</t>
+          <t>Attend the September SPARK initiative meeting</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -6800,12 +6800,12 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>September</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>End of August</t>
+          <t>End of September</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6821,7 +6821,7 @@
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -6835,17 +6835,17 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Implementation Q3</t>
+          <t>Implementation Q4</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Attend the September SPARK initiative meeting</t>
+          <t>Attend the October SPARK initiative meeting</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -6860,12 +6860,12 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>October</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>End of September</t>
+          <t>End of October</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6881,7 +6881,7 @@
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Attend the October SPARK initiative meeting</t>
+          <t>Attend the November SPARK initiative meeting</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -6920,12 +6920,12 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>November</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>End of October</t>
+          <t>End of November</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6941,7 +6941,7 @@
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -6965,7 +6965,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Attend the November SPARK initiative meeting</t>
+          <t>Attend the December SPARK initiative meeting</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -6980,12 +6980,12 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>November</t>
+          <t>December</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>End of November</t>
+          <t>End of December</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7001,11 +7001,11 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>SPARK</t>
+          <t>SOAR</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -7015,17 +7015,17 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Implementation Q4</t>
+          <t>Implementation Q1</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Attend the December SPARK initiative meeting</t>
+          <t>Attend the January SOAR initiative meeting</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -7040,12 +7040,12 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>December</t>
+          <t>January</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>End of December</t>
+          <t>End of January</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7061,7 +7061,7 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -7085,7 +7085,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Attend the January SOAR initiative meeting</t>
+          <t>Attend the February SOAR initiative meeting</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -7100,12 +7100,12 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>January</t>
+          <t>February</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>End of January</t>
+          <t>End of February</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7121,7 +7121,7 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -7145,7 +7145,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Attend the February SOAR initiative meeting</t>
+          <t>Attend the March SOAR initiative meeting</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -7160,12 +7160,12 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>February</t>
+          <t>March</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>End of February</t>
+          <t>End of March</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7181,7 +7181,7 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -7195,17 +7195,17 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Implementation Q1</t>
+          <t>Implementation Q2</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Attend the March SOAR initiative meeting</t>
+          <t>Attend the April SOAR initiative meeting</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -7220,12 +7220,12 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>March</t>
+          <t>April</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>End of March</t>
+          <t>End of April</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7241,7 +7241,7 @@
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -7265,7 +7265,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Attend the April SOAR initiative meeting</t>
+          <t>Attend the May SOAR initiative meeting</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -7280,12 +7280,12 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>April</t>
+          <t>May</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>End of April</t>
+          <t>End of May</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7301,7 +7301,7 @@
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -7325,7 +7325,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Attend the May SOAR initiative meeting</t>
+          <t>Attend the June SOAR initiative meeting</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -7340,12 +7340,12 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>June</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>End of May</t>
+          <t>End of June</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7361,7 +7361,7 @@
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -7375,17 +7375,17 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Implementation Q2</t>
+          <t>Implementation Q3</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Attend the June SOAR initiative meeting</t>
+          <t>Attend the July SOAR initiative meeting</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -7400,12 +7400,12 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>June</t>
+          <t>July</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>End of June</t>
+          <t>End of July</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7421,7 +7421,7 @@
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -7445,7 +7445,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Attend the July SOAR initiative meeting</t>
+          <t>Attend the August SOAR initiative meeting</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -7460,12 +7460,12 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>July</t>
+          <t>August</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>End of July</t>
+          <t>End of August</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7481,7 +7481,7 @@
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -7505,7 +7505,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Attend the August SOAR initiative meeting</t>
+          <t>Attend the September SOAR initiative meeting</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -7520,12 +7520,12 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>September</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>End of August</t>
+          <t>End of September</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7541,7 +7541,7 @@
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -7555,17 +7555,17 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Implementation Q3</t>
+          <t>Implementation Q4</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Attend the September SOAR initiative meeting</t>
+          <t>Attend the October SOAR initiative meeting</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -7580,12 +7580,12 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>October</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>End of September</t>
+          <t>End of October</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7601,7 +7601,7 @@
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Attend the October SOAR initiative meeting</t>
+          <t>Attend the November SOAR initiative meeting</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -7640,12 +7640,12 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>November</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>End of October</t>
+          <t>End of November</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7661,7 +7661,7 @@
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Attend the November SOAR initiative meeting</t>
+          <t>Attend the December SOAR initiative meeting</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -7700,12 +7700,12 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>November</t>
+          <t>December</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>End of November</t>
+          <t>End of December</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7721,11 +7721,11 @@
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>SOAR</t>
+          <t>NEST</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -7735,17 +7735,17 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Implementation Q4</t>
+          <t>Implementation Q1</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Attend the December SOAR initiative meeting</t>
+          <t>Attend the January NEST initiative meeting</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -7760,12 +7760,12 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>December</t>
+          <t>January</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>End of December</t>
+          <t>End of January</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7781,7 +7781,7 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -7805,7 +7805,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Attend the January NEST initiative meeting</t>
+          <t>Attend the February NEST initiative meeting</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -7820,12 +7820,12 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>January</t>
+          <t>February</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>End of January</t>
+          <t>End of February</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7841,7 +7841,7 @@
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Attend the February NEST initiative meeting</t>
+          <t>Attend the March NEST initiative meeting</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -7880,12 +7880,12 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>February</t>
+          <t>March</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>End of February</t>
+          <t>End of March</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7901,7 +7901,7 @@
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -7915,17 +7915,17 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Implementation Q1</t>
+          <t>Implementation Q2</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Attend the March NEST initiative meeting</t>
+          <t>Attend the April NEST initiative meeting</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -7940,12 +7940,12 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>March</t>
+          <t>April</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>End of March</t>
+          <t>End of April</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -7961,7 +7961,7 @@
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -7985,7 +7985,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Attend the April NEST initiative meeting</t>
+          <t>Attend the May NEST initiative meeting</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -8000,12 +8000,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>April</t>
+          <t>May</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>End of April</t>
+          <t>End of May</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8021,7 +8021,7 @@
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -8045,7 +8045,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Attend the May NEST initiative meeting</t>
+          <t>Attend the June NEST initiative meeting</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -8060,12 +8060,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>June</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>End of May</t>
+          <t>End of June</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8081,7 +8081,7 @@
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -8095,17 +8095,17 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Implementation Q2</t>
+          <t>Implementation Q3</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Attend the June NEST initiative meeting</t>
+          <t>Attend the July NEST initiative meeting</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -8120,12 +8120,12 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>June</t>
+          <t>July</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>End of June</t>
+          <t>End of July</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8141,7 +8141,7 @@
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -8165,7 +8165,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Attend the July NEST initiative meeting</t>
+          <t>Attend the August NEST initiative meeting</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -8180,12 +8180,12 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>July</t>
+          <t>August</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>End of July</t>
+          <t>End of August</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8201,7 +8201,7 @@
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -8225,7 +8225,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Attend the August NEST initiative meeting</t>
+          <t>Attend the September NEST initiative meeting</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -8240,12 +8240,12 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>September</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>End of August</t>
+          <t>End of September</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8261,7 +8261,7 @@
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -8275,17 +8275,17 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Implementation Q3</t>
+          <t>Implementation Q4</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Attend the September NEST initiative meeting</t>
+          <t>Attend the October NEST initiative meeting</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -8300,12 +8300,12 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>October</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>End of September</t>
+          <t>End of October</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8321,7 +8321,7 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -8345,7 +8345,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Attend the October NEST initiative meeting</t>
+          <t>Attend the November NEST initiative meeting</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -8360,12 +8360,12 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>November</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>End of October</t>
+          <t>End of November</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8381,7 +8381,7 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -8405,7 +8405,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Attend the November NEST initiative meeting</t>
+          <t>Attend the December NEST initiative meeting</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -8420,12 +8420,12 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>November</t>
+          <t>December</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>End of November</t>
+          <t>End of December</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8434,66 +8434,6 @@
         </is>
       </c>
       <c r="M127" t="inlineStr">
-        <is>
-          <t>Annual requirement: at least 9 of 12 monthly meetings. Annual Forum attendance counts toward the month it falls in (September in 2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="n">
-        <v>143</v>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>NEST</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>Implementation Q4</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>2.4</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>Attend the December NEST initiative meeting</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>meeting_attendance</t>
-        </is>
-      </c>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>December</t>
-        </is>
-      </c>
-      <c r="J128" t="inlineStr">
-        <is>
-          <t>End of December</t>
-        </is>
-      </c>
-      <c r="K128" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M128" t="inlineStr">
         <is>
           <t>Annual requirement: at least 9 of 12 monthly meetings. Annual Forum attendance counts toward the month it falls in (September in 2026).</t>
         </is>

</xml_diff>